<commit_message>
feat(report): split vendor portal bugs by phase
</commit_message>
<xml_diff>
--- a/fixtures/synthetic/odl-regression.xlsx
+++ b/fixtures/synthetic/odl-regression.xlsx
@@ -436,7 +436,7 @@
         <v>UAT-1</v>
       </c>
       <c r="B2" t="str">
-        <v>Subject 1</v>
+        <v>UAT Booking issue 1</v>
       </c>
       <c r="C2" t="str">
         <v>Bookings</v>
@@ -468,7 +468,7 @@
         <v>UAT-2</v>
       </c>
       <c r="B3" t="str">
-        <v>Subject 2</v>
+        <v>UAT Booking issue 2</v>
       </c>
       <c r="C3" t="str">
         <v>Bookings</v>
@@ -500,7 +500,7 @@
         <v>UAT-3</v>
       </c>
       <c r="B4" t="str">
-        <v>Subject 3</v>
+        <v>UAT Booking issue 3</v>
       </c>
       <c r="C4" t="str">
         <v>Bookings</v>
@@ -532,7 +532,7 @@
         <v>UAT-4</v>
       </c>
       <c r="B5" t="str">
-        <v>Subject 4</v>
+        <v>UAT Booking issue 4</v>
       </c>
       <c r="C5" t="str">
         <v>Bookings</v>
@@ -564,7 +564,7 @@
         <v>UAT-5</v>
       </c>
       <c r="B6" t="str">
-        <v>Subject 5</v>
+        <v>UAT Booking issue 5</v>
       </c>
       <c r="C6" t="str">
         <v>Bookings</v>
@@ -596,7 +596,7 @@
         <v>UAT-6</v>
       </c>
       <c r="B7" t="str">
-        <v>Subject 6</v>
+        <v>UAT Booking issue 6</v>
       </c>
       <c r="C7" t="str">
         <v>Bookings</v>
@@ -628,7 +628,7 @@
         <v>UAT-7</v>
       </c>
       <c r="B8" t="str">
-        <v>Subject 7</v>
+        <v>UAT Booking issue 7</v>
       </c>
       <c r="C8" t="str">
         <v>Bookings</v>
@@ -660,7 +660,7 @@
         <v>UAT-8</v>
       </c>
       <c r="B9" t="str">
-        <v>Subject 8</v>
+        <v>UAT Booking issue 8</v>
       </c>
       <c r="C9" t="str">
         <v>Bookings</v>
@@ -692,7 +692,7 @@
         <v>UAT-9</v>
       </c>
       <c r="B10" t="str">
-        <v>Subject 9</v>
+        <v>UAT Booking issue 9</v>
       </c>
       <c r="C10" t="str">
         <v>Bookings</v>
@@ -724,7 +724,7 @@
         <v>UAT-10</v>
       </c>
       <c r="B11" t="str">
-        <v>Subject 10</v>
+        <v>UAT Booking issue 10</v>
       </c>
       <c r="C11" t="str">
         <v>Bookings</v>
@@ -756,7 +756,7 @@
         <v>UAT-11</v>
       </c>
       <c r="B12" t="str">
-        <v>Subject 11</v>
+        <v>UAT Booking issue 11</v>
       </c>
       <c r="C12" t="str">
         <v>Bookings</v>
@@ -788,7 +788,7 @@
         <v>UAT-12</v>
       </c>
       <c r="B13" t="str">
-        <v>Subject 12</v>
+        <v>UAT Booking issue 12</v>
       </c>
       <c r="C13" t="str">
         <v>Bookings</v>
@@ -820,7 +820,7 @@
         <v>UAT-13</v>
       </c>
       <c r="B14" t="str">
-        <v>Subject 13</v>
+        <v>UAT Booking issue 13</v>
       </c>
       <c r="C14" t="str">
         <v>Bookings</v>
@@ -852,7 +852,7 @@
         <v>UAT-14</v>
       </c>
       <c r="B15" t="str">
-        <v>Subject 14</v>
+        <v>UAT Booking issue 14</v>
       </c>
       <c r="C15" t="str">
         <v>Bookings</v>
@@ -884,7 +884,7 @@
         <v>UAT-15</v>
       </c>
       <c r="B16" t="str">
-        <v>Subject 15</v>
+        <v>UAT Booking issue 15</v>
       </c>
       <c r="C16" t="str">
         <v>Bookings</v>
@@ -916,7 +916,7 @@
         <v>UAT-16</v>
       </c>
       <c r="B17" t="str">
-        <v>Subject 16</v>
+        <v>UAT Booking issue 16</v>
       </c>
       <c r="C17" t="str">
         <v>Bookings</v>
@@ -948,7 +948,7 @@
         <v>UAT-17</v>
       </c>
       <c r="B18" t="str">
-        <v>Subject 17</v>
+        <v>UAT Booking issue 17</v>
       </c>
       <c r="C18" t="str">
         <v>Bookings</v>
@@ -980,7 +980,7 @@
         <v>UAT-18</v>
       </c>
       <c r="B19" t="str">
-        <v>Subject 18</v>
+        <v>UAT Booking issue 18</v>
       </c>
       <c r="C19" t="str">
         <v>Bookings</v>
@@ -1012,7 +1012,7 @@
         <v>UAT-19</v>
       </c>
       <c r="B20" t="str">
-        <v>Subject 19</v>
+        <v>UAT Booking issue 19</v>
       </c>
       <c r="C20" t="str">
         <v>Bookings</v>
@@ -1044,7 +1044,7 @@
         <v>UAT-20</v>
       </c>
       <c r="B21" t="str">
-        <v>Subject 20</v>
+        <v>UAT Booking issue 20</v>
       </c>
       <c r="C21" t="str">
         <v>Bookings</v>
@@ -1076,7 +1076,7 @@
         <v>UAT-21</v>
       </c>
       <c r="B22" t="str">
-        <v>Subject 21</v>
+        <v>UAT Booking issue 21</v>
       </c>
       <c r="C22" t="str">
         <v>Bookings</v>
@@ -1108,7 +1108,7 @@
         <v>UAT-22</v>
       </c>
       <c r="B23" t="str">
-        <v>Subject 22</v>
+        <v>UAT Booking issue 22</v>
       </c>
       <c r="C23" t="str">
         <v>Bookings</v>
@@ -1140,7 +1140,7 @@
         <v>UAT-23</v>
       </c>
       <c r="B24" t="str">
-        <v>Subject 23</v>
+        <v>UAT Booking issue 23</v>
       </c>
       <c r="C24" t="str">
         <v>Bookings</v>
@@ -1172,7 +1172,7 @@
         <v>UAT-24</v>
       </c>
       <c r="B25" t="str">
-        <v>Subject 24</v>
+        <v>UAT Booking issue 24</v>
       </c>
       <c r="C25" t="str">
         <v>Bookings</v>
@@ -1204,7 +1204,7 @@
         <v>UAT-25</v>
       </c>
       <c r="B26" t="str">
-        <v>Subject 25</v>
+        <v>UAT Booking issue 25</v>
       </c>
       <c r="C26" t="str">
         <v>Bookings</v>
@@ -1236,7 +1236,7 @@
         <v>UAT-26</v>
       </c>
       <c r="B27" t="str">
-        <v>Subject 26</v>
+        <v>UAT Booking issue 26</v>
       </c>
       <c r="C27" t="str">
         <v>Bookings</v>
@@ -1268,7 +1268,7 @@
         <v>UAT-27</v>
       </c>
       <c r="B28" t="str">
-        <v>Subject 27</v>
+        <v>UAT Booking issue 27</v>
       </c>
       <c r="C28" t="str">
         <v>Bookings</v>
@@ -1300,7 +1300,7 @@
         <v>UAT-28</v>
       </c>
       <c r="B29" t="str">
-        <v>Subject 28</v>
+        <v>UAT Booking issue 28</v>
       </c>
       <c r="C29" t="str">
         <v>Bookings</v>
@@ -1332,7 +1332,7 @@
         <v>UAT-29</v>
       </c>
       <c r="B30" t="str">
-        <v>Subject 29</v>
+        <v>UAT Booking issue 29</v>
       </c>
       <c r="C30" t="str">
         <v>Bookings</v>
@@ -1364,7 +1364,7 @@
         <v>UAT-30</v>
       </c>
       <c r="B31" t="str">
-        <v>Subject 30</v>
+        <v>UAT Booking issue 30</v>
       </c>
       <c r="C31" t="str">
         <v>Bookings</v>
@@ -1396,7 +1396,7 @@
         <v>UAT-31</v>
       </c>
       <c r="B32" t="str">
-        <v>Subject 31</v>
+        <v>UAT Booking issue 31</v>
       </c>
       <c r="C32" t="str">
         <v>Bookings</v>
@@ -1428,7 +1428,7 @@
         <v>UAT-32</v>
       </c>
       <c r="B33" t="str">
-        <v>Subject 32</v>
+        <v>UAT Booking issue 32</v>
       </c>
       <c r="C33" t="str">
         <v>Bookings</v>
@@ -1460,7 +1460,7 @@
         <v>UAT-33</v>
       </c>
       <c r="B34" t="str">
-        <v>Subject 33</v>
+        <v>Phase 2B UAT Booking issue 33</v>
       </c>
       <c r="C34" t="str">
         <v>Bookings</v>
@@ -1492,7 +1492,7 @@
         <v>UAT-34</v>
       </c>
       <c r="B35" t="str">
-        <v>Subject 34</v>
+        <v>Phase 2B UAT Booking issue 34</v>
       </c>
       <c r="C35" t="str">
         <v>Bookings</v>
@@ -1524,7 +1524,7 @@
         <v>UAT-35</v>
       </c>
       <c r="B36" t="str">
-        <v>Subject 35</v>
+        <v>Phase 2B UAT Booking issue 35</v>
       </c>
       <c r="C36" t="str">
         <v>Bookings</v>
@@ -1556,7 +1556,7 @@
         <v>UAT-36</v>
       </c>
       <c r="B37" t="str">
-        <v>Subject 36</v>
+        <v>Phase 2B UAT Booking issue 36</v>
       </c>
       <c r="C37" t="str">
         <v>Bookings</v>
@@ -1588,7 +1588,7 @@
         <v>UAT-37</v>
       </c>
       <c r="B38" t="str">
-        <v>Subject 37</v>
+        <v>Phase 2B UAT Booking issue 37</v>
       </c>
       <c r="C38" t="str">
         <v>Bookings</v>
@@ -1620,7 +1620,7 @@
         <v>UAT-38</v>
       </c>
       <c r="B39" t="str">
-        <v>Subject 38</v>
+        <v>Phase 2B UAT Booking issue 38</v>
       </c>
       <c r="C39" t="str">
         <v>Bookings</v>
@@ -1652,7 +1652,7 @@
         <v>UAT-39</v>
       </c>
       <c r="B40" t="str">
-        <v>Subject 39</v>
+        <v>Phase 2B UAT Booking issue 39</v>
       </c>
       <c r="C40" t="str">
         <v>Bookings</v>
@@ -1684,7 +1684,7 @@
         <v>UAT-40</v>
       </c>
       <c r="B41" t="str">
-        <v>Subject 40</v>
+        <v>Phase 2B UAT Booking issue 40</v>
       </c>
       <c r="C41" t="str">
         <v>Bookings</v>
@@ -1716,7 +1716,7 @@
         <v>UAT-41</v>
       </c>
       <c r="B42" t="str">
-        <v>Subject 41</v>
+        <v>Phase 2B UAT Booking issue 41</v>
       </c>
       <c r="C42" t="str">
         <v>Bookings</v>
@@ -1748,7 +1748,7 @@
         <v>UAT-42</v>
       </c>
       <c r="B43" t="str">
-        <v>Subject 42</v>
+        <v>Phase 2B UAT Booking issue 42</v>
       </c>
       <c r="C43" t="str">
         <v>Bookings</v>
@@ -1780,7 +1780,7 @@
         <v>UAT-43</v>
       </c>
       <c r="B44" t="str">
-        <v>Subject 43</v>
+        <v>Phase 2B UAT Booking issue 43</v>
       </c>
       <c r="C44" t="str">
         <v>Bookings</v>
@@ -1812,7 +1812,7 @@
         <v>UAT-44</v>
       </c>
       <c r="B45" t="str">
-        <v>Subject 44</v>
+        <v>Phase 2B UAT Booking issue 44</v>
       </c>
       <c r="C45" t="str">
         <v>Bookings</v>
@@ -1844,7 +1844,7 @@
         <v>UAT-45</v>
       </c>
       <c r="B46" t="str">
-        <v>Subject 45</v>
+        <v>Phase 2B UAT Booking issue 45</v>
       </c>
       <c r="C46" t="str">
         <v>Bookings</v>
@@ -1876,7 +1876,7 @@
         <v>UAT-46</v>
       </c>
       <c r="B47" t="str">
-        <v>Subject 46</v>
+        <v>Phase 2B UAT Booking issue 46</v>
       </c>
       <c r="C47" t="str">
         <v>Bookings</v>
@@ -1908,7 +1908,7 @@
         <v>UAT-47</v>
       </c>
       <c r="B48" t="str">
-        <v>Subject 47</v>
+        <v>Phase 2B UAT Booking issue 47</v>
       </c>
       <c r="C48" t="str">
         <v>Bookings</v>
@@ -1940,7 +1940,7 @@
         <v>UAT-48</v>
       </c>
       <c r="B49" t="str">
-        <v>Subject 48</v>
+        <v>Phase 2B UAT Booking issue 48</v>
       </c>
       <c r="C49" t="str">
         <v>Bookings</v>
@@ -1972,7 +1972,7 @@
         <v>UAT-49</v>
       </c>
       <c r="B50" t="str">
-        <v>Subject 49</v>
+        <v>Phase 2B UAT Booking issue 49</v>
       </c>
       <c r="C50" t="str">
         <v>Bookings</v>
@@ -2004,7 +2004,7 @@
         <v>UAT-50</v>
       </c>
       <c r="B51" t="str">
-        <v>Subject 50</v>
+        <v>Phase 2B UAT Booking issue 50</v>
       </c>
       <c r="C51" t="str">
         <v>Bookings</v>
@@ -2036,7 +2036,7 @@
         <v>UAT-51</v>
       </c>
       <c r="B52" t="str">
-        <v>Subject 51</v>
+        <v>Phase 2B UAT Booking issue 51</v>
       </c>
       <c r="C52" t="str">
         <v>Bookings</v>
@@ -2068,7 +2068,7 @@
         <v>UAT-52</v>
       </c>
       <c r="B53" t="str">
-        <v>Subject 52</v>
+        <v>Phase 2B UAT Booking issue 52</v>
       </c>
       <c r="C53" t="str">
         <v>Bookings</v>
@@ -2100,7 +2100,7 @@
         <v>UAT-53</v>
       </c>
       <c r="B54" t="str">
-        <v>Subject 53</v>
+        <v>Phase 2B UAT Booking issue 53</v>
       </c>
       <c r="C54" t="str">
         <v>Bookings</v>
@@ -2132,7 +2132,7 @@
         <v>UAT-54</v>
       </c>
       <c r="B55" t="str">
-        <v>Subject 54</v>
+        <v>Phase 2B UAT Booking issue 54</v>
       </c>
       <c r="C55" t="str">
         <v>Bookings</v>
@@ -2164,7 +2164,7 @@
         <v>UAT-55</v>
       </c>
       <c r="B56" t="str">
-        <v>Subject 55</v>
+        <v>INC000055 Production issue 55</v>
       </c>
       <c r="C56" t="str">
         <v>Bookings</v>
@@ -2196,7 +2196,7 @@
         <v>UAT-56</v>
       </c>
       <c r="B57" t="str">
-        <v>Subject 56</v>
+        <v>INC000056 Production issue 56</v>
       </c>
       <c r="C57" t="str">
         <v>Bookings</v>
@@ -2228,7 +2228,7 @@
         <v>UAT-57</v>
       </c>
       <c r="B58" t="str">
-        <v>Subject 57</v>
+        <v>INC000057 Production issue 57</v>
       </c>
       <c r="C58" t="str">
         <v>Bookings</v>
@@ -2260,7 +2260,7 @@
         <v>UAT-58</v>
       </c>
       <c r="B59" t="str">
-        <v>Subject 58</v>
+        <v>INC000058 Production issue 58</v>
       </c>
       <c r="C59" t="str">
         <v>Bookings</v>
@@ -2292,7 +2292,7 @@
         <v>UAT-59</v>
       </c>
       <c r="B60" t="str">
-        <v>Subject 59</v>
+        <v>INC000059 Production issue 59</v>
       </c>
       <c r="C60" t="str">
         <v>Bookings</v>
@@ -2324,7 +2324,7 @@
         <v>UAT-60</v>
       </c>
       <c r="B61" t="str">
-        <v>Subject 60</v>
+        <v>INC000060 Production issue 60</v>
       </c>
       <c r="C61" t="str">
         <v>Bookings</v>
@@ -2356,7 +2356,7 @@
         <v>UAT-61</v>
       </c>
       <c r="B62" t="str">
-        <v>Subject 61</v>
+        <v>INC000061 Production issue 61</v>
       </c>
       <c r="C62" t="str">
         <v>Bookings</v>
@@ -2388,7 +2388,7 @@
         <v>UAT-62</v>
       </c>
       <c r="B63" t="str">
-        <v>Subject 62</v>
+        <v>INC000062 Production issue 62</v>
       </c>
       <c r="C63" t="str">
         <v>Bookings</v>
@@ -2420,7 +2420,7 @@
         <v>UAT-63</v>
       </c>
       <c r="B64" t="str">
-        <v>Subject 63</v>
+        <v>INC000063 Production issue 63</v>
       </c>
       <c r="C64" t="str">
         <v>Bookings</v>
@@ -2452,7 +2452,7 @@
         <v>UAT-64</v>
       </c>
       <c r="B65" t="str">
-        <v>Subject 64</v>
+        <v>INC000064 Production issue 64</v>
       </c>
       <c r="C65" t="str">
         <v>Bookings</v>
@@ -2484,7 +2484,7 @@
         <v>UAT-65</v>
       </c>
       <c r="B66" t="str">
-        <v>Subject 65</v>
+        <v>INC000065 Production issue 65</v>
       </c>
       <c r="C66" t="str">
         <v>Bookings</v>
@@ -2516,7 +2516,7 @@
         <v>UAT-66</v>
       </c>
       <c r="B67" t="str">
-        <v>Subject 66</v>
+        <v>INC000066 Production issue 66</v>
       </c>
       <c r="C67" t="str">
         <v>Bookings</v>
@@ -2548,7 +2548,7 @@
         <v>UAT-67</v>
       </c>
       <c r="B68" t="str">
-        <v>Subject 67</v>
+        <v>INC000067 Production issue 67</v>
       </c>
       <c r="C68" t="str">
         <v>Bookings</v>
@@ -2580,7 +2580,7 @@
         <v>UAT-68</v>
       </c>
       <c r="B69" t="str">
-        <v>Subject 68</v>
+        <v>INC000068 Production issue 68</v>
       </c>
       <c r="C69" t="str">
         <v>Bookings</v>
@@ -2612,7 +2612,7 @@
         <v>UAT-69</v>
       </c>
       <c r="B70" t="str">
-        <v>Subject 69</v>
+        <v>INC000069 Production issue 69</v>
       </c>
       <c r="C70" t="str">
         <v>Bookings</v>
@@ -2644,7 +2644,7 @@
         <v>UAT-70</v>
       </c>
       <c r="B71" t="str">
-        <v>Subject 70</v>
+        <v>INC000070 Production issue 70</v>
       </c>
       <c r="C71" t="str">
         <v>Bookings</v>
@@ -2676,7 +2676,7 @@
         <v>UAT-71</v>
       </c>
       <c r="B72" t="str">
-        <v>Subject 71</v>
+        <v>Booking issue without prefix 71</v>
       </c>
       <c r="C72" t="str">
         <v>Bookings</v>
@@ -2708,7 +2708,7 @@
         <v>UAT-72</v>
       </c>
       <c r="B73" t="str">
-        <v>Subject 72</v>
+        <v>Booking issue without prefix 72</v>
       </c>
       <c r="C73" t="str">
         <v>Bookings</v>
@@ -2740,7 +2740,7 @@
         <v>UAT-73</v>
       </c>
       <c r="B74" t="str">
-        <v>Subject 73</v>
+        <v>Booking issue without prefix 73</v>
       </c>
       <c r="C74" t="str">
         <v>Bookings</v>
@@ -2772,7 +2772,7 @@
         <v>UAT-74</v>
       </c>
       <c r="B75" t="str">
-        <v>Subject 74</v>
+        <v>Booking issue without prefix 74</v>
       </c>
       <c r="C75" t="str">
         <v>Bookings</v>

</xml_diff>